<commit_message>
api response updates ,api array input change ,
</commit_message>
<xml_diff>
--- a/batch_test_results.xlsx
+++ b/batch_test_results.xlsx
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bluebird Group LLC, The</t>
+          <t>Aechelon Technology Inc.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -501,12 +501,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Bluebird</t>
+          <t>Aechelon</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bluebird</t>
+          <t>Aechelon</t>
         </is>
       </c>
       <c r="F2" t="b">
@@ -514,12 +514,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Bluebird (Term Loan)</t>
+          <t>Aechelon (Term Loan)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Bluebird (Term Loan)</t>
+          <t>Aechelon (Term Loan)</t>
         </is>
       </c>
       <c r="I2" t="b">
@@ -543,7 +543,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Events Buyer, LLC</t>
+          <t>BlueHalo Global Holdings, LLC</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -553,17 +553,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>360DG</t>
+          <t>BlueHalo</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>360DG</t>
+          <t>BlueHalo</t>
         </is>
       </c>
       <c r="F3" t="b">
@@ -571,12 +571,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>360DG (Term Loan)</t>
+          <t>BlueHalo (Term Loan)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>360DG (Term Loan)</t>
+          <t>BlueHalo (Term Loan)</t>
         </is>
       </c>
       <c r="I3" t="b">
@@ -600,7 +600,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Burgess Point Purchaser Corporation</t>
+          <t>Bluebird Group LLC, The</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -610,17 +610,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>BBB Industries</t>
+          <t>Bluebird</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BBB Industries</t>
+          <t>Bluebird</t>
         </is>
       </c>
       <c r="F4" t="b">
@@ -628,12 +628,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>BBB Industries (First Lien Term Loan)</t>
+          <t>Bluebird (Term Loan)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>BBB Industries (First Lien Term Loan)</t>
+          <t>Bluebird (Term Loan)</t>
         </is>
       </c>
       <c r="I4" t="b">
@@ -657,7 +657,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>48forty Intermediate Holdings, Inc.</t>
+          <t>Ad.net Acquisition, LLC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -672,12 +672,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>48Forty</t>
+          <t>Ad.net</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>48Forty</t>
+          <t>Ad.net</t>
         </is>
       </c>
       <c r="F5" t="b">
@@ -685,12 +685,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>48Forty (Common Equity)</t>
+          <t>Ad.net (Term Loan)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>48Forty (Common Equity)</t>
+          <t>Ad.net (Term Loan)</t>
         </is>
       </c>
       <c r="I5" t="b">
@@ -714,7 +714,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Aegis Technologies Group, LLC, The</t>
+          <t>BLC Holding Company, Inc.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -729,12 +729,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>BlueHalo</t>
+          <t>Bland Landscaping</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BlueHalo</t>
+          <t>Bland Landscaping</t>
         </is>
       </c>
       <c r="F6" t="b">
@@ -742,12 +742,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>BlueHalo (Term Loan)</t>
+          <t>Bland Landscaping (DDTL)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>BlueHalo (Term Loan)</t>
+          <t>Bland Landscaping (DDTL)</t>
         </is>
       </c>
       <c r="I6" t="b">
@@ -771,7 +771,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ad.net Acquisition, LLC</t>
+          <t>AFC-Dell Holding Corp.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -781,17 +781,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Knowledge Match</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Ad.net</t>
+          <t>AFC Acquisitions</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Ad.net</t>
+          <t>AFC Acquisitions</t>
         </is>
       </c>
       <c r="F7" t="b">
@@ -799,12 +799,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Ad.net (Term Loan)</t>
+          <t>AFC Industries (DDTL)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Ad.net (Term Loan)</t>
+          <t>AFC Industries (DDTL)</t>
         </is>
       </c>
       <c r="I7" t="b">
@@ -828,7 +828,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AFC-Dell Holding Corp.</t>
+          <t>Burgess Point Purchaser Corporation</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -838,17 +838,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Company Knowledge Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>AFC Acquisitions</t>
+          <t>BBB Industries</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AFC Acquisitions</t>
+          <t>BBB Industries</t>
         </is>
       </c>
       <c r="F8" t="b">
@@ -856,12 +856,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>AFC Industries (TL)</t>
+          <t>BBB Industries (First Lien Term Loan)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>AFC Industries (TL)</t>
+          <t>BBB Industries (First Lien Term Loan)</t>
         </is>
       </c>
       <c r="I8" t="b">
@@ -885,7 +885,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AFC-Dell Holding Corp.</t>
+          <t>By Light Professional IT Services LLC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -895,17 +895,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Company Knowledge Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AFC Acquisitions</t>
+          <t>By Light</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AFC Acquisitions</t>
+          <t>By Light</t>
         </is>
       </c>
       <c r="F9" t="b">
@@ -913,12 +913,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>AFC Industries (DDTL)</t>
+          <t>By Light (Revolver)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>AFC Industries (DDTL)</t>
+          <t>By Light (Revolver)</t>
         </is>
       </c>
       <c r="I9" t="b">
@@ -942,7 +942,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Aechelon Technology Inc.</t>
+          <t>Aegis Technologies Group, LLC, The</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -952,17 +952,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Aechelon</t>
+          <t>BlueHalo</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Aechelon</t>
+          <t>BlueHalo</t>
         </is>
       </c>
       <c r="F10" t="b">
@@ -970,12 +970,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Aechelon (Term Loan)</t>
+          <t>BlueHalo (Term Loan)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Aechelon (Term Loan)</t>
+          <t>BlueHalo (Term Loan)</t>
         </is>
       </c>
       <c r="I10" t="b">
@@ -999,7 +999,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>By Light Professional IT Services LLC</t>
+          <t>AFC-Dell Holding Corp.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1009,17 +1009,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Knowledge Match</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>By Light</t>
+          <t>AFC Acquisitions</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>By Light</t>
+          <t>AFC Acquisitions</t>
         </is>
       </c>
       <c r="F11" t="b">
@@ -1027,12 +1027,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>By Light (Revolver)</t>
+          <t>AFC Industries (TL)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>By Light (Revolver)</t>
+          <t>AFC Industries (TL)</t>
         </is>
       </c>
       <c r="I11" t="b">
@@ -1056,7 +1056,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BlueHalo Global Holdings, LLC</t>
+          <t>Events Buyer, LLC</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1066,17 +1066,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>BlueHalo</t>
+          <t>360DG</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BlueHalo</t>
+          <t>360DG</t>
         </is>
       </c>
       <c r="F12" t="b">
@@ -1084,12 +1084,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>BlueHalo (Term Loan)</t>
+          <t>360DG (Term Loan)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>BlueHalo (Term Loan)</t>
+          <t>360DG (Term Loan)</t>
         </is>
       </c>
       <c r="I12" t="b">
@@ -1113,7 +1113,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dr. Squatch, LLC</t>
+          <t>48forty Intermediate Holdings, Inc.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1128,12 +1128,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Dr. Squatch</t>
+          <t>48Forty</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Dr. Squatch</t>
+          <t>48Forty</t>
         </is>
       </c>
       <c r="F13" t="b">
@@ -1141,12 +1141,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Dr. Squatch (Term Loan)</t>
+          <t>48Forty (Common Equity)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Dr. Squatch (Term Loan)</t>
+          <t>48Forty (Common Equity)</t>
         </is>
       </c>
       <c r="I13" t="b">
@@ -1170,7 +1170,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GGG Midco, LLC</t>
+          <t>Dr. Squatch, LLC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1180,17 +1180,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Guild Garage Group</t>
+          <t>Dr. Squatch</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Guild Garage Group</t>
+          <t>Dr. Squatch</t>
         </is>
       </c>
       <c r="F14" t="b">
@@ -1198,12 +1198,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Guild Garage Group (DDTL)</t>
+          <t>Dr. Squatch (Term Loan)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Guild Garage Group (DDTL)</t>
+          <t>Dr. Squatch (Term Loan)</t>
         </is>
       </c>
       <c r="I14" t="b">
@@ -1227,7 +1227,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Lash Opco, LLC</t>
+          <t>Infinity Home Services Holdco, Inc</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1237,17 +1237,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Lilly Lashes</t>
+          <t>Infinity Home Services</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Lilly Lashes</t>
+          <t>Infinity Home Services</t>
         </is>
       </c>
       <c r="F15" t="b">
@@ -1255,12 +1255,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Lilly Lashes (TL)</t>
+          <t>Infinity Home Services (DDTL)</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Lilly Lashes (TL)</t>
+          <t>Infinity Home Services (DDTL)</t>
         </is>
       </c>
       <c r="I15" t="b">
@@ -1284,7 +1284,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Infinity Home Services Holdco, Inc</t>
+          <t>GGG Midco, LLC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1294,17 +1294,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Infinity Home Services</t>
+          <t>Guild Garage Group</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Infinity Home Services</t>
+          <t>Guild Garage Group</t>
         </is>
       </c>
       <c r="F16" t="b">
@@ -1312,12 +1312,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Infinity Home Services (DDTL)</t>
+          <t>Guild Garage Group (DDTL)</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Infinity Home Services (DDTL)</t>
+          <t>Guild Garage Group (DDTL)</t>
         </is>
       </c>
       <c r="I16" t="b">
@@ -1341,7 +1341,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>OSP EMBEDDED PURCHASER, LLC</t>
+          <t>Lash Opco, LLC</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1356,12 +1356,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Lynx Technologies</t>
+          <t>Lilly Lashes</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Lynx Technologies</t>
+          <t>Lilly Lashes</t>
         </is>
       </c>
       <c r="F17" t="b">
@@ -1369,12 +1369,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Lynx Technologies (TL)</t>
+          <t>Lilly Lashes (TL)</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Lynx Technologies (TL)</t>
+          <t>Lilly Lashes (TL)</t>
         </is>
       </c>
       <c r="I17" t="b">
@@ -1455,7 +1455,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MeritDirect, LLC</t>
+          <t>OSP EMBEDDED PURCHASER, LLC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1465,17 +1465,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MeritDirect</t>
+          <t>Lynx Technologies</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MeritDirect</t>
+          <t>Lynx Technologies</t>
         </is>
       </c>
       <c r="F19" t="b">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>MeritDirect (Term Loan)</t>
+          <t>Lynx Technologies (TL)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>MeritDirect (Term Loan)</t>
+          <t>Lynx Technologies (TL)</t>
         </is>
       </c>
       <c r="I19" t="b">
@@ -1512,7 +1512,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pragmatic Institute, LLC</t>
+          <t>MeritDirect, LLC</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1527,12 +1527,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Pragmatic Institute</t>
+          <t>MeritDirect</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Pragmatic Institute</t>
+          <t>MeritDirect</t>
         </is>
       </c>
       <c r="F20" t="b">
@@ -1540,12 +1540,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Pragmatic Institute (Common)</t>
+          <t>MeritDirect (Term Loan)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Pragmatic Institute (Common)</t>
+          <t>MeritDirect (Term Loan)</t>
         </is>
       </c>
       <c r="I20" t="b">
@@ -1569,7 +1569,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Paving Lessor Corp.</t>
+          <t>Pragmatic Institute, LLC</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1579,17 +1579,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>C&amp;K Paving Contractors</t>
+          <t>Pragmatic Institute</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>C&amp;K Paving Contractors</t>
+          <t>Pragmatic Institute</t>
         </is>
       </c>
       <c r="F21" t="b">
@@ -1597,12 +1597,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>C&amp;K Paving Contractors (Term Loan)</t>
+          <t>Pragmatic Institute (Common)</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>C&amp;K Paving Contractors (Term Loan)</t>
+          <t>Pragmatic Institute (Common)</t>
         </is>
       </c>
       <c r="I21" t="b">
@@ -1626,7 +1626,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Lightspeed Buyer, Inc.</t>
+          <t>Paving Lessor Corp.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1641,25 +1641,29 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Centauri Health</t>
+          <t>C&amp;K Paving Contractors</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Centauri Health</t>
+          <t>C&amp;K Paving Contractors</t>
         </is>
       </c>
       <c r="F22" t="b">
         <v>1</v>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>C&amp;K Paving Contractors (Term Loan)</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Centauri Health (TL)</t>
+          <t>C&amp;K Paving Contractors (Term Loan)</t>
         </is>
       </c>
       <c r="I22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1679,7 +1683,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NFS - CFP Holdings LLC</t>
+          <t>Lightspeed Buyer, Inc.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1694,12 +1698,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Commercial Fire Protection</t>
+          <t>Centauri Health</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Commercial Fire Protection</t>
+          <t>Centauri Health</t>
         </is>
       </c>
       <c r="F23" t="b">
@@ -1707,12 +1711,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Commercial Fire Protection (Term Loan)</t>
+          <t>Centauri Health (TL)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Commercial Fire Protection (Term Loan)</t>
+          <t>Centauri Health (TL)</t>
         </is>
       </c>
       <c r="I23" t="b">
@@ -1736,7 +1740,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DRS Holdings III, Inc.</t>
+          <t>NFS - CFP Holdings LLC</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1751,12 +1755,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Dr. Scholl's</t>
+          <t>Commercial Fire Protection</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Dr. Scholl's</t>
+          <t>Commercial Fire Protection</t>
         </is>
       </c>
       <c r="F24" t="b">
@@ -1764,12 +1768,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Dr. Scholl's (Term Loan)</t>
+          <t>Commercial Fire Protection (Term Loan)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Dr. Scholl's (Term Loan)</t>
+          <t>Commercial Fire Protection (Term Loan)</t>
         </is>
       </c>
       <c r="I24" t="b">
@@ -1793,7 +1797,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Management Consulting &amp; Research, LLC</t>
+          <t>DRS Holdings III, Inc.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1808,12 +1812,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>MCR</t>
+          <t>Dr. Scholl's</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MCR</t>
+          <t>Dr. Scholl's</t>
         </is>
       </c>
       <c r="F25" t="b">
@@ -1821,12 +1825,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>MCR (Term Loan)</t>
+          <t>Dr. Scholl's (Term Loan)</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>MCR (Term Loan)</t>
+          <t>Dr. Scholl's (Term Loan)</t>
         </is>
       </c>
       <c r="I25" t="b">
@@ -1850,7 +1854,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PlayPower, Inc.</t>
+          <t>Management Consulting &amp; Research, LLC</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1860,17 +1864,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>PlayPower</t>
+          <t>MCR</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>PlayPower</t>
+          <t>MCR</t>
         </is>
       </c>
       <c r="F26" t="b">
@@ -1878,12 +1882,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>PlayPower (Term Loan)</t>
+          <t>MCR (Term Loan)</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>PlayPower (Term Loan)</t>
+          <t>MCR (Term Loan)</t>
         </is>
       </c>
       <c r="I26" t="b">
@@ -1907,27 +1911,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>48Forty Intermediate Holdings Inc</t>
+          <t>Arcline FM Holdings LLC</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>watc_holdings</t>
+          <t>us bank cashfile</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Knowledge Match</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>48Forty</t>
+          <t>Fairbanks Morse Defense</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>48Forty</t>
+          <t>Fairbanks Morse Defense</t>
         </is>
       </c>
       <c r="F27" t="b">
@@ -1935,12 +1939,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>48Forty (Common Equity)</t>
+          <t>Fairbanks Morse Defense (Term Loan)</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>48Forty (Common Equity)</t>
+          <t>Fairbanks Morse Defense (Term Loan)</t>
         </is>
       </c>
       <c r="I27" t="b">
@@ -1964,27 +1968,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LAV Gear Holdings Inc</t>
+          <t>PlayPower, Inc.</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>watc_holdings</t>
+          <t>us bank cashfile</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>4Wall Entertainment</t>
+          <t>PlayPower</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>4Wall Entertainment</t>
+          <t>PlayPower</t>
         </is>
       </c>
       <c r="F28" t="b">
@@ -1992,12 +1996,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>4Wall Entertainment (Term Loan)</t>
+          <t>PlayPower (Term Loan)</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>4Wall Entertainment (Term Loan)</t>
+          <t>PlayPower (Term Loan)</t>
         </is>
       </c>
       <c r="I28" t="b">
@@ -2021,27 +2025,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Burgess Point Purchaser Corporation</t>
+          <t>The Track Branson Opco, LLC</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>watc_holdings</t>
+          <t>us bank cashfile</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Company Knowledge Match</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>BBB Industries</t>
+          <t>The Creative Group</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>BBB Industries</t>
+          <t>The Creative Group</t>
         </is>
       </c>
       <c r="F29" t="b">
@@ -2049,12 +2053,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>BBB Industries (First Lien Term Loan)</t>
+          <t>The Creative Group (Term Loan)</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>BBB Industries (First Lien Term Loan)</t>
+          <t>The Creative Group (Term Loan)</t>
         </is>
       </c>
       <c r="I29" t="b">
@@ -2078,12 +2082,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Big Top Holdings LLC</t>
+          <t>Lightspeed Buyer, Inc.</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>watc_holdings</t>
+          <t>us bank cashfile</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2093,12 +2097,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Big Top Manufacturing</t>
+          <t>Centauri Health</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Big Top Manufacturing</t>
+          <t>Centauri Health</t>
         </is>
       </c>
       <c r="F30" t="b">
@@ -2106,20 +2110,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Big Top Manufacturing (Term Loan)</t>
+          <t>Centauri Health (Revolver)</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Big Top Manufacturing (Term Loan)</t>
+          <t>Centauri Health (TL)</t>
         </is>
       </c>
       <c r="I30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K30" t="b">
@@ -2135,7 +2139,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BlueHalo Global Holdings LLC</t>
+          <t>48Forty Intermediate Holdings Inc</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2150,12 +2154,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>BlueHalo</t>
+          <t>48Forty</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>BlueHalo</t>
+          <t>48Forty</t>
         </is>
       </c>
       <c r="F31" t="b">
@@ -2163,12 +2167,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>BlueHalo (Term Loan)</t>
+          <t>48Forty (Common Equity)</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>BlueHalo (Term Loan)</t>
+          <t>48Forty (Common Equity)</t>
         </is>
       </c>
       <c r="I31" t="b">
@@ -2192,12 +2196,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Lightspeed Buyer, Inc.</t>
+          <t>LAV Gear Holdings Inc</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>us bank cashfile</t>
+          <t>watc_holdings</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2207,12 +2211,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Centauri Health</t>
+          <t>4Wall Entertainment</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Centauri Health</t>
+          <t>4Wall Entertainment</t>
         </is>
       </c>
       <c r="F32" t="b">
@@ -2220,20 +2224,20 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Centauri Health (Revolver)</t>
+          <t>4Wall Entertainment (Term Loan)</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Centauri Health (TL)</t>
+          <t>4Wall Entertainment (Term Loan)</t>
         </is>
       </c>
       <c r="I32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="K32" t="b">
@@ -2249,7 +2253,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ACP Falcon Buyer Inc</t>
+          <t>Sath Industries LLC</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2259,17 +2263,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Company Knowledge Match</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Integrated Data Services</t>
+          <t>360DG</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Integrated Data Services</t>
+          <t>360DG</t>
         </is>
       </c>
       <c r="F33" t="b">
@@ -2277,12 +2281,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Integrated Data Services (TL)</t>
+          <t>360DG (DDTL A)</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Integrated Data Services (TL)</t>
+          <t>360DG (DDTL A)</t>
         </is>
       </c>
       <c r="I33" t="b">
@@ -2306,7 +2310,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Kinetic Purchaser LLC</t>
+          <t>Burgess Point Purchaser Corporation</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2321,12 +2325,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>KNS</t>
+          <t>BBB Industries</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>KNS</t>
+          <t>BBB Industries</t>
         </is>
       </c>
       <c r="F34" t="b">
@@ -2334,12 +2338,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>KNS (Term Loan)</t>
+          <t>BBB Industries (First Lien Term Loan)</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>KNS (Term Loan)</t>
+          <t>BBB Industries (First Lien Term Loan)</t>
         </is>
       </c>
       <c r="I34" t="b">
@@ -2363,27 +2367,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OSG Topco Holdings LLC - Class A Unit</t>
+          <t>Big Top Holdings LLC</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>us bank cashfile</t>
+          <t>watc_holdings</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>OSG Billing Services</t>
+          <t>Big Top Manufacturing</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>OSG Billing Services</t>
+          <t>Big Top Manufacturing</t>
         </is>
       </c>
       <c r="F35" t="b">
@@ -2391,20 +2395,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>OSG (Common Equity)</t>
+          <t>Big Top Manufacturing (Term Loan)</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>U.S. Well (Class A)</t>
+          <t>Big Top Manufacturing (Term Loan)</t>
         </is>
       </c>
       <c r="I35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="K35" t="b">
@@ -2420,12 +2424,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Radius Aerospace Inc</t>
+          <t>OSG Topco Holdings LLC - Class A Unit</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>watc_holdings</t>
+          <t>us bank cashfile</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2435,33 +2439,33 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Radius Aerospace</t>
+          <t>OSG Billing Services</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Radius Aerospace</t>
+          <t>U.S. Well</t>
         </is>
       </c>
       <c r="F36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Radius Aerospace (Term Loan)</t>
+          <t>OSG (Common Equity)</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Radius Aerospace (Term Loan)</t>
+          <t>U.S. Well (Class A)</t>
         </is>
       </c>
       <c r="I36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K36" t="b">
@@ -2477,7 +2481,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>RRA Corporate LLC</t>
+          <t>BlueHalo Global Holdings LLC</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2487,17 +2491,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Roofed Right America</t>
+          <t>BlueHalo</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Roofed Right America</t>
+          <t>BlueHalo</t>
         </is>
       </c>
       <c r="F37" t="b">
@@ -2505,12 +2509,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Roofed Right America (Term Loan)</t>
+          <t>BlueHalo (Term Loan)</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Roofed Right America (Term Loan)</t>
+          <t>BlueHalo (Term Loan)</t>
         </is>
       </c>
       <c r="I37" t="b">
@@ -2534,48 +2538,48 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Arcline FM Holdings LLC</t>
+          <t>ACP Falcon Buyer Inc</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>us bank cashfile</t>
+          <t>watc_holdings</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Company Knowledge Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Fairbanks Morse Defense</t>
+          <t>Integrated Data Services</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>AKW Holdings</t>
+          <t>Integrated Data Services</t>
         </is>
       </c>
       <c r="F38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Fairbanks Morse Defense (Term Loan)</t>
+          <t>Integrated Data Services (TL)</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>AKW Holdings (Term Loan)</t>
+          <t>Integrated Data Services (TL)</t>
         </is>
       </c>
       <c r="I38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="K38" t="b">
@@ -2591,7 +2595,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DRS Holdings III Inc</t>
+          <t>Kinetic Purchaser LLC</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2606,12 +2610,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Dr. Scholl's</t>
+          <t>KNS</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Dr. Scholl's</t>
+          <t>KNS</t>
         </is>
       </c>
       <c r="F39" t="b">
@@ -2619,12 +2623,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Dr. Scholl's (Term Loan)</t>
+          <t>KNS (Term Loan)</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Dr. Scholl's (Term Loan)</t>
+          <t>KNS (Term Loan)</t>
         </is>
       </c>
       <c r="I39" t="b">
@@ -2648,7 +2652,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Systems Planning and Analysis Inc</t>
+          <t>Radius Aerospace Inc</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2658,17 +2662,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Company Knowledge Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>MCR</t>
+          <t>Radius Aerospace</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>MCR</t>
+          <t>Radius Aerospace</t>
         </is>
       </c>
       <c r="F40" t="b">
@@ -2676,12 +2680,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>MCR (Term Loan)</t>
+          <t>Radius Aerospace (Term Loan)</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>MCR (Term Loan)</t>
+          <t>Radius Aerospace (Term Loan)</t>
         </is>
       </c>
       <c r="I40" t="b">
@@ -2705,48 +2709,48 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>The Track Branson Opco, LLC</t>
+          <t>RRA Corporate LLC</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>us bank cashfile</t>
+          <t>watc_holdings</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Company Knowledge Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>The Creative Group</t>
+          <t>Roofed Right America</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>APT Healthcare</t>
+          <t>Roofed Right America</t>
         </is>
       </c>
       <c r="F41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>The Creative Group (Term Loan)</t>
+          <t>Roofed Right America (Term Loan)</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>APT Healthcare (Incr. DDTL)</t>
+          <t>Roofed Right America (Term Loan)</t>
         </is>
       </c>
       <c r="I41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="K41" t="b">
@@ -2762,7 +2766,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Sath Industries LLC</t>
+          <t>TMII Enterprises LLC</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2777,33 +2781,33 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>360DG</t>
+          <t>A1 Garage</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Boss Industries</t>
+          <t>A1 Garage</t>
         </is>
       </c>
       <c r="F42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>360DG (DDTL A)</t>
+          <t>A1 Garage (DDTL)</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>AFC Industries (DDTL)</t>
+          <t>A1 Garage (DDTL)</t>
         </is>
       </c>
       <c r="I42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="K42" t="b">
@@ -2819,7 +2823,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>STG Distribution LLC</t>
+          <t>TMII Enterprises LLC</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2829,17 +2833,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Knowledge Match</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>STG Logistics</t>
+          <t>A1 Garage</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>STG Logistics</t>
+          <t>A1 Garage</t>
         </is>
       </c>
       <c r="F43" t="b">
@@ -2847,12 +2851,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>STG (First Out New Money Term Loans)</t>
+          <t>A1 Garage (Term Loan)</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>STG (First Out New Money Term Loans)</t>
+          <t>A1 Garage (Term Loan)</t>
         </is>
       </c>
       <c r="I43" t="b">
@@ -2933,27 +2937,27 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>LAV Gear Holdings, Inc.</t>
+          <t>Systems Planning and Analysis Inc</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>market_value</t>
+          <t>watc_holdings</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Company Knowledge Match</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>4Wall Entertainment</t>
+          <t>MCR</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>4Wall Entertainment</t>
+          <t>MCR</t>
         </is>
       </c>
       <c r="F45" t="b">
@@ -2961,12 +2965,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>4Wall Entertainment (Term Loan)</t>
+          <t>MCR (Term Loan)</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>4Wall Entertainment (Term Loan)</t>
+          <t>MCR (Term Loan)</t>
         </is>
       </c>
       <c r="I45" t="b">
@@ -2990,27 +2994,27 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>A1 Garage Equity, LLC</t>
+          <t>DRS Holdings III Inc</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>market_value</t>
+          <t>watc_holdings</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>A1 Garage</t>
+          <t>Dr. Scholl's</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>A1 Garage</t>
+          <t>Dr. Scholl's</t>
         </is>
       </c>
       <c r="F46" t="b">
@@ -3018,12 +3022,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>A1 Garage (Common Equity)</t>
+          <t>Dr. Scholl's (Term Loan)</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>A1 Garage (Common Equity)</t>
+          <t>Dr. Scholl's (Term Loan)</t>
         </is>
       </c>
       <c r="I46" t="b">
@@ -3047,27 +3051,27 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Archer Lewis, LLC</t>
+          <t>SMX Group LLC</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>market_value</t>
+          <t>watc_holdings</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Knowledge Match</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Archer Lewis</t>
+          <t>Smartronix / Trident</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Archer Lewis</t>
+          <t>Smartronix / Trident</t>
         </is>
       </c>
       <c r="F47" t="b">
@@ -3075,12 +3079,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Archer Lewis (Revolver)</t>
+          <t>Smartronix / Trident (TL)</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Archer Lewis (Revolver)</t>
+          <t>Smartronix / Trident (TL)</t>
         </is>
       </c>
       <c r="I47" t="b">
@@ -3104,12 +3108,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Beta Plus Technologies, Inc.</t>
+          <t>STG Distribution LLC</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>market_value</t>
+          <t>watc_holdings</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3119,12 +3123,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Beta+</t>
+          <t>STG Logistics</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Beta+</t>
+          <t>STG Logistics</t>
         </is>
       </c>
       <c r="F48" t="b">
@@ -3132,12 +3136,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Beta+ (TL)</t>
+          <t>STG (First Out New Money Term Loans)</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Beta+ (TL)</t>
+          <t>STG (First Out New Money Term Loans)</t>
         </is>
       </c>
       <c r="I48" t="b">
@@ -3161,7 +3165,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Rural Sourcing Holdings, Inc.</t>
+          <t>LAV Gear Holdings, Inc.</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3171,17 +3175,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Company Knowledge Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Sparq</t>
+          <t>4Wall Entertainment</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Sparq</t>
+          <t>4Wall Entertainment</t>
         </is>
       </c>
       <c r="F49" t="b">
@@ -3189,12 +3193,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Sparq (TL)</t>
+          <t>4Wall Entertainment (Term Loan)</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Sparq (TL)</t>
+          <t>4Wall Entertainment (Term Loan)</t>
         </is>
       </c>
       <c r="I49" t="b">
@@ -3218,7 +3222,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TCG 3.0 Jogger Acquisitionco, Inc.</t>
+          <t>A1 Garage Equity, LLC</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3228,17 +3232,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>BiggerPockets</t>
+          <t>A1 Garage</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>BiggerPockets</t>
+          <t>A1 Garage</t>
         </is>
       </c>
       <c r="F50" t="b">
@@ -3246,12 +3250,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>BiggerPockets (Revolver)</t>
+          <t>A1 Garage (Common Equity)</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>BiggerPockets (Revolver)</t>
+          <t>A1 Garage (Common Equity)</t>
         </is>
       </c>
       <c r="I50" t="b">
@@ -3275,7 +3279,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Carnegie Dartlet, LLC</t>
+          <t>Archer Lewis, LLC</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3290,12 +3294,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Carnegie Dartlet</t>
+          <t>Archer Lewis</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Carnegie Dartlet</t>
+          <t>Archer Lewis</t>
         </is>
       </c>
       <c r="F51" t="b">
@@ -3303,12 +3307,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Carnegie Dartlet (DDTL)</t>
+          <t>Archer Lewis (Revolver)</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Carnegie Dartlet (DDTL)</t>
+          <t>Archer Lewis (Revolver)</t>
         </is>
       </c>
       <c r="I51" t="b">
@@ -3332,48 +3336,48 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>TMII Enterprises LLC</t>
+          <t>Beta Plus Technologies, Inc.</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>watc_holdings</t>
+          <t>market_value</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Company Knowledge Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>A1 Garage</t>
+          <t>Beta+</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>TVC</t>
+          <t>Beta+</t>
         </is>
       </c>
       <c r="F52" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>A1 Garage (DDTL)</t>
+          <t>Beta+ (TL)</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>US Fertility (DDTL)</t>
+          <t>Beta+ (TL)</t>
         </is>
       </c>
       <c r="I52" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="K52" t="b">
@@ -3389,7 +3393,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Medina Health, LLC</t>
+          <t>Rural Sourcing Holdings, Inc.</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3399,17 +3403,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Company Knowledge Match</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Comprehensive Rehab Consultants</t>
+          <t>Sparq</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Comprehensive Rehab Consultants</t>
+          <t>Sparq</t>
         </is>
       </c>
       <c r="F53" t="b">
@@ -3417,12 +3421,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Comprehensive Rehab Consultants (Revolver)</t>
+          <t>Sparq (TL)</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Comprehensive Rehab Consultants (Revolver)</t>
+          <t>Sparq (TL)</t>
         </is>
       </c>
       <c r="I53" t="b">
@@ -3446,7 +3450,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>GAUGE ETE BLOCKER LLC</t>
+          <t>TCG 3.0 Jogger Acquisitionco, Inc.</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3461,12 +3465,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Engine &amp; Transmission Exchange</t>
+          <t>BiggerPockets</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Engine &amp; Transmission Exchange</t>
+          <t>BiggerPockets</t>
         </is>
       </c>
       <c r="F54" t="b">
@@ -3474,12 +3478,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Engine &amp; Transmission Exchange (Common Equity)</t>
+          <t>BiggerPockets (Revolver)</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Engine &amp; Transmission Exchange (Common Equity)</t>
+          <t>BiggerPockets (Revolver)</t>
         </is>
       </c>
       <c r="I54" t="b">
@@ -3503,27 +3507,27 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SV-Aero Holdings LLC</t>
+          <t>Carnegie Dartlet, LLC</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>watc_holdings</t>
+          <t>market_value</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Company Knowledge Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Aeronix</t>
+          <t>Carnegie Dartlet</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Aeronix</t>
+          <t>Carnegie Dartlet</t>
         </is>
       </c>
       <c r="F55" t="b">
@@ -3531,20 +3535,20 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Aeronix (TL)</t>
+          <t>Carnegie Dartlet (DDTL)</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Aeronix (DDTL)</t>
+          <t>Carnegie Dartlet (DDTL)</t>
         </is>
       </c>
       <c r="I55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="K55" t="b">
@@ -3560,7 +3564,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>EDS TOPCO, LP</t>
+          <t>Medina Health, LLC</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3575,12 +3579,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Epiq</t>
+          <t>Comprehensive Rehab Consultants</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Epiq</t>
+          <t>Comprehensive Rehab Consultants</t>
         </is>
       </c>
       <c r="F56" t="b">
@@ -3588,12 +3592,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Epiq (Common)</t>
+          <t>Comprehensive Rehab Consultants (Revolver)</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Epiq (Common)</t>
+          <t>Comprehensive Rehab Consultants (Revolver)</t>
         </is>
       </c>
       <c r="I56" t="b">
@@ -3617,7 +3621,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ENC Parent Corporation</t>
+          <t>GAUGE ETE BLOCKER LLC</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3632,12 +3636,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Evans Network</t>
+          <t>Engine &amp; Transmission Exchange</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Evans Network</t>
+          <t>Engine &amp; Transmission Exchange</t>
         </is>
       </c>
       <c r="F57" t="b">
@@ -3645,12 +3649,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Evans Network (1L)</t>
+          <t>Engine &amp; Transmission Exchange (Common Equity)</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Evans Network (1L)</t>
+          <t>Engine &amp; Transmission Exchange (Common Equity)</t>
         </is>
       </c>
       <c r="I57" t="b">
@@ -3674,7 +3678,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Best Practice Associates, LLC</t>
+          <t>ENC Parent Corporation</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3689,12 +3693,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Federal Advisory Partners</t>
+          <t>Evans Network</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Federal Advisory Partners</t>
+          <t>Evans Network</t>
         </is>
       </c>
       <c r="F58" t="b">
@@ -3702,12 +3706,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Federal Advisory Partners (First Lien Term Loan)</t>
+          <t>Evans Network (1L)</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Federal Advisory Partners (First Lien Term Loan)</t>
+          <t>Evans Network (1L)</t>
         </is>
       </c>
       <c r="I58" t="b">
@@ -3731,7 +3735,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Infinity Home Services Holdco, Inc.</t>
+          <t>EDS TOPCO, LP</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3741,17 +3745,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Infinity Home Services</t>
+          <t>Epiq</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Infinity Home Services</t>
+          <t>Epiq</t>
         </is>
       </c>
       <c r="F59" t="b">
@@ -3759,12 +3763,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Infinity Home Services (Revolver)</t>
+          <t>Epiq (Common)</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Infinity Home Services (Revolver)</t>
+          <t>Epiq (Common)</t>
         </is>
       </c>
       <c r="I59" t="b">
@@ -3788,7 +3792,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SMX Group LLC</t>
+          <t>SV-Aero Holdings LLC</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3803,25 +3807,25 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Smartronix / Trident</t>
+          <t>Aeronix</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Simplicity Group</t>
+          <t>Aeronix</t>
         </is>
       </c>
       <c r="F60" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Smartronix / Trident (TL)</t>
+          <t>Aeronix (TL)</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>STV Group (TL)</t>
+          <t>Aeronix (DDTL)</t>
         </is>
       </c>
       <c r="I60" t="b">
@@ -3845,27 +3849,27 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Zips Car Wash LLC</t>
+          <t>Best Practice Associates, LLC</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>watc_holdings</t>
+          <t>market_value</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Zips</t>
+          <t>Federal Advisory Partners</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Zips</t>
+          <t>Federal Advisory Partners</t>
         </is>
       </c>
       <c r="F61" t="b">
@@ -3873,20 +3877,20 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Zips (Rollup DIP Term Loan)</t>
+          <t>Federal Advisory Partners (First Lien Term Loan)</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Zips (Term Loan)</t>
+          <t>Federal Advisory Partners (First Lien Term Loan)</t>
         </is>
       </c>
       <c r="I61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="K61" t="b">
@@ -3902,48 +3906,48 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>TMII Enterprises LLC</t>
+          <t>Infinity Home Services Holdco, Inc.</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>watc_holdings</t>
+          <t>market_value</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Company Knowledge Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>A1 Garage</t>
+          <t>Infinity Home Services</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>TVC</t>
+          <t>Infinity Home Services</t>
         </is>
       </c>
       <c r="F62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>A1 Garage (Term Loan)</t>
+          <t>Infinity Home Services (Revolver)</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>TVC (TL)</t>
+          <t>Infinity Home Services (Revolver)</t>
         </is>
       </c>
       <c r="I62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="K62" t="b">
@@ -3959,27 +3963,27 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Dr. Scholl's</t>
+          <t>Zips Car Wash LLC</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>master_ratings</t>
+          <t>watc_holdings</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Dr. Scholl's</t>
+          <t>Zips</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Dr. Scholl's</t>
+          <t>Zips</t>
         </is>
       </c>
       <c r="F63" t="b">
@@ -3987,20 +3991,20 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Dr. Scholl's (Revolver)</t>
+          <t>Zips (Rollup DIP Term Loan)</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Dr. Scholl's (Revolver)</t>
+          <t>Zips (Term Loan)</t>
         </is>
       </c>
       <c r="I63" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K63" t="b">
@@ -4016,7 +4020,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Recteq</t>
+          <t>Dr. Scholl's</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -4031,12 +4035,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Recteq</t>
+          <t>Dr. Scholl's</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Recteq</t>
+          <t>Dr. Scholl's</t>
         </is>
       </c>
       <c r="F64" t="b">
@@ -4044,12 +4048,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Recteq (Equity)</t>
+          <t>Dr. Scholl's (Revolver)</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Recteq (Equity)</t>
+          <t>Dr. Scholl's (Revolver)</t>
         </is>
       </c>
       <c r="I64" t="b">
@@ -4073,27 +4077,27 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>HV Watterson Holdings, LLC</t>
+          <t>Recteq</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>consolidated_soi</t>
+          <t>master_ratings</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Watterson</t>
+          <t>Recteq</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Watterson</t>
+          <t>Recteq</t>
         </is>
       </c>
       <c r="F65" t="b">
@@ -4101,12 +4105,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Watterson (Revolver)</t>
+          <t>Recteq (Equity)</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Watterson (Revolver)</t>
+          <t>Recteq (Equity)</t>
         </is>
       </c>
       <c r="I65" t="b">
@@ -4130,7 +4134,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Watchtower Buyer, LLC</t>
+          <t>HV Watterson Holdings, LLC</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -4145,12 +4149,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Watchtower Buyer</t>
+          <t>Watterson</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Watchtower Buyer</t>
+          <t>Watterson</t>
         </is>
       </c>
       <c r="F66" t="b">
@@ -4158,12 +4162,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Watchtower Buyer (Revolver)</t>
+          <t>Watterson (Revolver)</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Watchtower Buyer (Revolver)</t>
+          <t>Watterson (Revolver)</t>
         </is>
       </c>
       <c r="I66" t="b">
@@ -4187,12 +4191,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Aeronix</t>
+          <t>MidOcean JF Holdings Corp.</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>master_ratings</t>
+          <t>market_value</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -4202,12 +4206,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Aeronix</t>
+          <t>Jones &amp; Frank</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Aeronix</t>
+          <t>Jones &amp; Frank</t>
         </is>
       </c>
       <c r="F67" t="b">
@@ -4215,12 +4219,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Aeronix (Common Equity)</t>
+          <t>Jones &amp; Frank (TL)</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Aeronix (Revolver)</t>
+          <t>Jones &amp; Frank (Common)</t>
         </is>
       </c>
       <c r="I67" t="b">
@@ -4244,12 +4248,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>MidOcean JF Holdings Corp.</t>
+          <t>4Wall Entertainment</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>market_value</t>
+          <t>master_ratings</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -4259,12 +4263,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Jones &amp; Frank</t>
+          <t>4Wall Entertainment</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Jones &amp; Frank</t>
+          <t>4Wall Entertainment</t>
         </is>
       </c>
       <c r="F68" t="b">
@@ -4272,12 +4276,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Jones &amp; Frank (TL)</t>
+          <t>4Wall Entertainment (Term Loan)</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Jones &amp; Frank (Common)</t>
+          <t>4Wall Entertainment (Revolver)</t>
         </is>
       </c>
       <c r="I68" t="b">
@@ -4301,7 +4305,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Any Hour Services</t>
+          <t>Aeronix</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4316,12 +4320,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Any Hour Services</t>
+          <t>Aeronix</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Any Hour Services</t>
+          <t>Aeronix</t>
         </is>
       </c>
       <c r="F69" t="b">
@@ -4329,12 +4333,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Any Hour Services (DDTL II)</t>
+          <t>Aeronix (Common Equity)</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Any Hour Services (Revolver)</t>
+          <t>Aeronix (Revolver)</t>
         </is>
       </c>
       <c r="I69" t="b">
@@ -4358,27 +4362,27 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Any Hour Services</t>
+          <t>Watchtower Buyer, LLC</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>master_ratings</t>
+          <t>consolidated_soi</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Any Hour Services</t>
+          <t>Watchtower Buyer</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Any Hour Services</t>
+          <t>Watchtower Buyer</t>
         </is>
       </c>
       <c r="F70" t="b">
@@ -4386,20 +4390,20 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Any Hour Services (Common Equity)</t>
+          <t>Watchtower Buyer (Revolver)</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Any Hour Services (Revolver)</t>
+          <t>Watchtower Buyer (Revolver)</t>
         </is>
       </c>
       <c r="I70" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="K70" t="b">
@@ -4415,7 +4419,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Cano Health</t>
+          <t>Any Hour Services</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -4430,12 +4434,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Cano Health</t>
+          <t>Any Hour Services</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Cano Health</t>
+          <t>Any Hour Services</t>
         </is>
       </c>
       <c r="F71" t="b">
@@ -4443,16 +4447,16 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Cano Health (Equity)</t>
+          <t>Any Hour Services (Common Equity)</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Cano Health (Equity)</t>
+          <t>Any Hour Services (Revolver)</t>
         </is>
       </c>
       <c r="I71" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J71" t="inlineStr">
         <is>
@@ -4472,27 +4476,27 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>UniVista Insurance</t>
+          <t>Any Hour Services</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>consolidated_soi</t>
+          <t>master_ratings</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>UniVista</t>
+          <t>Any Hour Services</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>UniVista</t>
+          <t>Any Hour Services</t>
         </is>
       </c>
       <c r="F72" t="b">
@@ -4500,20 +4504,20 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>UniVista (Equity)</t>
+          <t>Any Hour Services (DDTL II)</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>UniVista (Equity)</t>
+          <t>Any Hour Services (Revolver)</t>
         </is>
       </c>
       <c r="I72" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K72" t="b">
@@ -4529,12 +4533,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Project Granite Buyer, Inc.</t>
+          <t>Cano Health</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>consolidated_soi</t>
+          <t>master_ratings</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -4544,12 +4548,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Tranzact</t>
+          <t>Cano Health</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Tranzact</t>
+          <t>Cano Health</t>
         </is>
       </c>
       <c r="F73" t="b">
@@ -4557,12 +4561,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Tranzact (Term Loan)</t>
+          <t>Cano Health (Equity)</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Tranzact (Term Loan)</t>
+          <t>Cano Health (Equity)</t>
         </is>
       </c>
       <c r="I73" t="b">
@@ -4570,7 +4574,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>direct</t>
         </is>
       </c>
       <c r="K73" t="b">
@@ -4586,7 +4590,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>TransGo, LLC</t>
+          <t>UniVista Insurance</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4596,17 +4600,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>TransGo</t>
+          <t>UniVista</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>TransGo</t>
+          <t>UniVista</t>
         </is>
       </c>
       <c r="F74" t="b">
@@ -4614,12 +4618,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>TransGo (Equity)</t>
+          <t>UniVista (Equity)</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>TransGo (Equity)</t>
+          <t>UniVista (Equity)</t>
         </is>
       </c>
       <c r="I74" t="b">
@@ -4643,7 +4647,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Infinity Home Services</t>
+          <t>KNS</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -4658,12 +4662,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Infinity Home Services</t>
+          <t>KNS</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Infinity Home Services</t>
+          <t>KNS</t>
         </is>
       </c>
       <c r="F75" t="b">
@@ -4671,12 +4675,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Infinity Home Services (DDTL)</t>
+          <t>KNS (Term Loan)</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Infinity Home Services (Revolver)</t>
+          <t>KNS (Equity)</t>
         </is>
       </c>
       <c r="I75" t="b">
@@ -4700,7 +4704,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>STG Distribution, LLC</t>
+          <t>Project Granite Buyer, Inc.</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4710,17 +4714,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>STG Logistics</t>
+          <t>Tranzact</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>STG Logistics</t>
+          <t>Tranzact</t>
         </is>
       </c>
       <c r="F76" t="b">
@@ -4728,12 +4732,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>STG (Second Out Term Loans)</t>
+          <t>Tranzact (Term Loan)</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>STG (Second Out Term Loans)</t>
+          <t>Tranzact (Term Loan)</t>
         </is>
       </c>
       <c r="I76" t="b">
@@ -4757,7 +4761,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>KNS</t>
+          <t>Infinity Home Services</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4772,12 +4776,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>KNS</t>
+          <t>Infinity Home Services</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>KNS</t>
+          <t>Infinity Home Services</t>
         </is>
       </c>
       <c r="F77" t="b">
@@ -4785,12 +4789,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>KNS (Term Loan)</t>
+          <t>Infinity Home Services (DDTL)</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>KNS (Equity)</t>
+          <t>Infinity Home Services (Revolver)</t>
         </is>
       </c>
       <c r="I77" t="b">
@@ -4814,12 +4818,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>4Wall Entertainment</t>
+          <t>TransGo, LLC</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>master_ratings</t>
+          <t>consolidated_soi</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -4829,12 +4833,12 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>4Wall Entertainment</t>
+          <t>TransGo</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>4Wall Entertainment</t>
+          <t>TransGo</t>
         </is>
       </c>
       <c r="F78" t="b">
@@ -4842,20 +4846,20 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>4Wall Entertainment (Term Loan)</t>
+          <t>TransGo (Equity)</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>4Wall Entertainment (Revolver)</t>
+          <t>TransGo (Equity)</t>
         </is>
       </c>
       <c r="I78" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="K78" t="b">
@@ -4871,7 +4875,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Schlesinger Global, Inc.</t>
+          <t>STG Distribution, LLC</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4881,17 +4885,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Schlesinger</t>
+          <t>STG Logistics</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Schlesinger</t>
+          <t>STG Logistics</t>
         </is>
       </c>
       <c r="F79" t="b">
@@ -4899,12 +4903,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Schlesinger (Equity)</t>
+          <t>STG (Second Out Term Loans)</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Schlesinger (Equity)</t>
+          <t>STG (Second Out Term Loans)</t>
         </is>
       </c>
       <c r="I79" t="b">
@@ -4928,7 +4932,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Pacific Purchaser, LLC</t>
+          <t>Schlesinger Global, Inc.</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4943,12 +4947,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>ProSearch</t>
+          <t>Schlesinger</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>ProSearch</t>
+          <t>Schlesinger</t>
         </is>
       </c>
       <c r="F80" t="b">
@@ -4956,12 +4960,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>ProSearch (Revolver)</t>
+          <t>Schlesinger (Equity)</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>ProSearch (Revolver)</t>
+          <t>Schlesinger (Equity)</t>
         </is>
       </c>
       <c r="I80" t="b">
@@ -5042,12 +5046,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>TCG 3.0 Jogger Co-Invest, LP - Common Equity</t>
+          <t>Pacific Purchaser, LLC</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>daily_long_short</t>
+          <t>consolidated_soi</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -5057,12 +5061,12 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>BiggerPockets</t>
+          <t>ProSearch</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>BiggerPockets</t>
+          <t>ProSearch</t>
         </is>
       </c>
       <c r="F82" t="b">
@@ -5070,12 +5074,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>BiggerPockets (Common Equity)</t>
+          <t>ProSearch (Revolver)</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>BiggerPockets (Common Equity)</t>
+          <t>ProSearch (Revolver)</t>
         </is>
       </c>
       <c r="I82" t="b">
@@ -5099,7 +5103,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Knexus Holdco, LLC - Preferred Equity</t>
+          <t>TCG 3.0 Jogger Co-Invest, LP - Common Equity</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -5109,17 +5113,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Company Knowledge Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>C5MI</t>
+          <t>BiggerPockets</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>C5MI</t>
+          <t>BiggerPockets</t>
         </is>
       </c>
       <c r="F83" t="b">
@@ -5127,12 +5131,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>C5MI (Preferred Equity)</t>
+          <t>BiggerPockets (Common Equity)</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>C5MI (Preferred Equity)</t>
+          <t>BiggerPockets (Common Equity)</t>
         </is>
       </c>
       <c r="I83" t="b">
@@ -5156,7 +5160,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Connatix Parent, LLC - Common Equity</t>
+          <t>Knexus Holdco, LLC - Preferred Equity</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -5166,17 +5170,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Knowledge Match</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Connatix</t>
+          <t>C5MI</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Connatix</t>
+          <t>C5MI</t>
         </is>
       </c>
       <c r="F84" t="b">
@@ -5184,12 +5188,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Connatix (Common Equity)</t>
+          <t>C5MI (Preferred Equity)</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Connatix (Common Equity)</t>
+          <t>C5MI (Preferred Equity)</t>
         </is>
       </c>
       <c r="I84" t="b">
@@ -5213,7 +5217,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Connatix Parent, LLC - Preferred Equity</t>
+          <t>Connatix Parent, LLC - Common Equity</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -5270,7 +5274,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>RFMG Parent, LP - Common Equity</t>
+          <t>Connatix Parent, LLC - Preferred Equity</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -5280,17 +5284,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Rancho Medical</t>
+          <t>Connatix</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Rancho Medical</t>
+          <t>Connatix</t>
         </is>
       </c>
       <c r="F86" t="b">
@@ -5298,12 +5302,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Rancho (Equity)</t>
+          <t>Connatix (Common Equity)</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Rancho (Equity)</t>
+          <t>Connatix (Common Equity)</t>
         </is>
       </c>
       <c r="I86" t="b">
@@ -5327,7 +5331,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Project Granite Holdings, LLC - Common Equity</t>
+          <t>RFMG Parent, LP - Common Equity</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -5342,12 +5346,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Tranzact</t>
+          <t>Rancho Medical</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Tranzact</t>
+          <t>Rancho Medical</t>
         </is>
       </c>
       <c r="F87" t="b">
@@ -5355,12 +5359,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Tranzact (Common Equity)</t>
+          <t>Rancho (Equity)</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Tranzact (Common Equity)</t>
+          <t>Rancho (Equity)</t>
         </is>
       </c>
       <c r="I87" t="b">
@@ -5384,7 +5388,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>NXOF Holdings, Inc. - Common Equity</t>
+          <t>Project Granite Holdings, LLC - Common Equity</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -5399,12 +5403,12 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Tyto Athene</t>
+          <t>Tranzact</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Tyto Athene</t>
+          <t>Tranzact</t>
         </is>
       </c>
       <c r="F88" t="b">
@@ -5412,12 +5416,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Tyto Athene (Equity)</t>
+          <t>Tranzact (Common Equity)</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Tyto Athene (Equity)</t>
+          <t>Tranzact (Common Equity)</t>
         </is>
       </c>
       <c r="I88" t="b">
@@ -5555,7 +5559,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>TWD Parent Holdings, LLC - Preferred Equity</t>
+          <t>NXOF Holdings, Inc. - Common Equity</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -5570,12 +5574,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Tyto Athene</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Tyto Athene</t>
         </is>
       </c>
       <c r="F91" t="b">
@@ -5583,12 +5587,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Vertex (Preferred Equity)</t>
+          <t>Tyto Athene (Equity)</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Vertex (Preferred Equity)</t>
+          <t>Tyto Athene (Equity)</t>
         </is>
       </c>
       <c r="I91" t="b">
@@ -5612,7 +5616,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Watchtower Holdings, LLC - Common Equity</t>
+          <t>TWD Parent Holdings, LLC - Preferred Equity</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -5622,30 +5626,30 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Security Match</t>
+          <t>Company Match</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Watchtower</t>
+          <t>Vertex</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Watchtower Holdings</t>
+          <t>Vertex</t>
         </is>
       </c>
       <c r="F92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Watchtower Holding (Common Equity)</t>
+          <t>Vertex (Preferred Equity)</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Watchtower Holding (Common Equity)</t>
+          <t>Vertex (Preferred Equity)</t>
         </is>
       </c>
       <c r="I92" t="b">
@@ -5726,27 +5730,27 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Rural Sourcing Holdings, Inc.</t>
+          <t>Watchtower Holdings, LLC - Common Equity</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>consolidated_soi</t>
+          <t>daily_long_short</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Company Knowledge Match</t>
+          <t>Security Match</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Sparq</t>
+          <t>Watchtower Holdings</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Sparq</t>
+          <t>Watchtower Holdings</t>
         </is>
       </c>
       <c r="F94" t="b">
@@ -5754,20 +5758,20 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Sparq (Revolver)</t>
+          <t>Watchtower Holding (Common Equity)</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Sparq (TL)</t>
+          <t>Watchtower Holding (Common Equity)</t>
         </is>
       </c>
       <c r="I94" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="K94" t="b">
@@ -5783,47 +5787,59 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>BLC Holding Company, Inc.</t>
+          <t>Rural Sourcing Holdings, Inc.</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>us bank cashfile</t>
+          <t>consolidated_soi</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Company Match</t>
+          <t>Company Knowledge Match</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Bland Landscaping</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
+          <t>Sparq</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Sparq</t>
+        </is>
+      </c>
+      <c r="F95" t="b">
+        <v>1</v>
+      </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Bland Landscaping (DDTL)</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr"/>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
+          <t>Sparq (Revolver)</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Sparq (TL)</t>
+        </is>
+      </c>
+      <c r="I95" t="b">
+        <v>0</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
       <c r="K95" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="M95" t="inlineStr">
-        <is>
-          <t>HTTPConnectionPool(host='localhost', port=7071): Read timed out. (read timeout=10)</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>